<commit_message>
feat: Add educational resources on quality management, Lean Six Sigma, Pareto, and Ishikawa diagrams.
</commit_message>
<xml_diff>
--- a/OI/LEAN SS/frise historique industrie.xlsx
+++ b/OI/LEAN SS/frise historique industrie.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/Bachelor/2025 BACH/MA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cfaicentre-my.sharepoint.com/personal/s_jaubert_poleformation-uimmcvdl_fr/Documents/00FC/OI/LEAN SS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{BEB8309D-2044-4FA8-9699-538A31EB241A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6FFDFE1-CCDB-4234-8EB1-69FEEC58B57B}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{BEB8309D-2044-4FA8-9699-538A31EB241A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D9B7894-6A82-4D42-BDE5-8528AACC13E8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{06AFAFDD-76BD-492E-BDC8-55604D5A30B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{06AFAFDD-76BD-492E-BDC8-55604D5A30B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -1143,96 +1143,94 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1583,103 +1581,103 @@
   <sheetData>
     <row r="1" spans="1:83" s="5" customFormat="1" ht="64.900000000000006" customHeight="1" thickBot="1">
       <c r="A1" s="4"/>
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="66" t="s">
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="55" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="63" t="s">
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
+      <c r="N1" s="56"/>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="R1" s="64"/>
-      <c r="S1" s="64"/>
-      <c r="T1" s="64"/>
-      <c r="U1" s="64"/>
-      <c r="V1" s="64"/>
-      <c r="W1" s="64"/>
-      <c r="X1" s="64"/>
-      <c r="Y1" s="64"/>
-      <c r="Z1" s="64"/>
-      <c r="AA1" s="64"/>
-      <c r="AB1" s="63" t="s">
+      <c r="R1" s="58"/>
+      <c r="S1" s="58"/>
+      <c r="T1" s="58"/>
+      <c r="U1" s="58"/>
+      <c r="V1" s="58"/>
+      <c r="W1" s="58"/>
+      <c r="X1" s="58"/>
+      <c r="Y1" s="58"/>
+      <c r="Z1" s="58"/>
+      <c r="AA1" s="58"/>
+      <c r="AB1" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="AC1" s="64"/>
-      <c r="AD1" s="64"/>
-      <c r="AE1" s="64"/>
-      <c r="AF1" s="64"/>
-      <c r="AG1" s="64"/>
-      <c r="AH1" s="64"/>
-      <c r="AI1" s="64"/>
-      <c r="AJ1" s="64"/>
-      <c r="AK1" s="64"/>
-      <c r="AL1" s="64"/>
-      <c r="AM1" s="63" t="s">
+      <c r="AC1" s="58"/>
+      <c r="AD1" s="58"/>
+      <c r="AE1" s="58"/>
+      <c r="AF1" s="58"/>
+      <c r="AG1" s="58"/>
+      <c r="AH1" s="58"/>
+      <c r="AI1" s="58"/>
+      <c r="AJ1" s="58"/>
+      <c r="AK1" s="58"/>
+      <c r="AL1" s="58"/>
+      <c r="AM1" s="57" t="s">
         <v>85</v>
       </c>
-      <c r="AN1" s="64"/>
-      <c r="AO1" s="64"/>
-      <c r="AP1" s="64"/>
-      <c r="AQ1" s="64"/>
-      <c r="AR1" s="64"/>
-      <c r="AS1" s="64"/>
-      <c r="AT1" s="64"/>
-      <c r="AU1" s="64"/>
-      <c r="AV1" s="64"/>
-      <c r="AW1" s="64"/>
-      <c r="AX1" s="46" t="s">
+      <c r="AN1" s="58"/>
+      <c r="AO1" s="58"/>
+      <c r="AP1" s="58"/>
+      <c r="AQ1" s="58"/>
+      <c r="AR1" s="58"/>
+      <c r="AS1" s="58"/>
+      <c r="AT1" s="58"/>
+      <c r="AU1" s="58"/>
+      <c r="AV1" s="58"/>
+      <c r="AW1" s="58"/>
+      <c r="AX1" s="71" t="s">
         <v>86</v>
       </c>
-      <c r="AY1" s="47"/>
-      <c r="AZ1" s="47"/>
-      <c r="BA1" s="47"/>
-      <c r="BB1" s="47"/>
-      <c r="BC1" s="47"/>
-      <c r="BD1" s="47"/>
-      <c r="BE1" s="47"/>
-      <c r="BF1" s="47"/>
-      <c r="BG1" s="47"/>
-      <c r="BH1" s="47"/>
+      <c r="AY1" s="72"/>
+      <c r="AZ1" s="72"/>
+      <c r="BA1" s="72"/>
+      <c r="BB1" s="72"/>
+      <c r="BC1" s="72"/>
+      <c r="BD1" s="72"/>
+      <c r="BE1" s="72"/>
+      <c r="BF1" s="72"/>
+      <c r="BG1" s="72"/>
+      <c r="BH1" s="72"/>
     </row>
     <row r="2" spans="1:83" s="14" customFormat="1" ht="99.75" customHeight="1" thickBot="1">
       <c r="A2" s="16"/>
       <c r="B2" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="65" t="s">
+      <c r="C2" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="65"/>
+      <c r="D2" s="59"/>
       <c r="E2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="65" t="s">
+      <c r="F2" s="59" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-      <c r="J2" s="65"/>
-      <c r="K2" s="65"/>
-      <c r="L2" s="65"/>
-      <c r="M2" s="65"/>
-      <c r="N2" s="65"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="65"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
       <c r="Q2" s="19" t="s">
         <v>8</v>
       </c>
@@ -1692,10 +1690,10 @@
         <v>10</v>
       </c>
       <c r="AB2" s="17"/>
-      <c r="AK2" s="65" t="s">
+      <c r="AK2" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="AL2" s="65"/>
+      <c r="AL2" s="59"/>
       <c r="AM2" s="14" t="s">
         <v>12</v>
       </c>
@@ -1736,19 +1734,19 @@
       <c r="C3" s="43"/>
       <c r="D3" s="43"/>
       <c r="E3" s="15"/>
-      <c r="F3" s="69" t="s">
+      <c r="F3" s="61" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="70"/>
-      <c r="H3" s="70"/>
-      <c r="I3" s="70"/>
-      <c r="J3" s="70"/>
-      <c r="K3" s="70"/>
-      <c r="L3" s="70"/>
-      <c r="M3" s="70"/>
-      <c r="N3" s="70"/>
-      <c r="O3" s="70"/>
-      <c r="P3" s="71"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="62"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="63"/>
       <c r="Q3" s="15"/>
       <c r="R3" s="15"/>
       <c r="S3" s="15"/>
@@ -1760,44 +1758,44 @@
       <c r="Y3" s="15"/>
       <c r="Z3" s="15"/>
       <c r="AA3" s="15"/>
-      <c r="AB3" s="49" t="s">
+      <c r="AB3" s="64" t="s">
         <v>16</v>
       </c>
-      <c r="AC3" s="49"/>
-      <c r="AD3" s="49"/>
-      <c r="AE3" s="49"/>
-      <c r="AF3" s="49"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="64"/>
+      <c r="AE3" s="64"/>
+      <c r="AF3" s="64"/>
       <c r="AG3" s="15"/>
       <c r="AH3" s="15"/>
       <c r="AI3" s="15"/>
       <c r="AJ3" s="15"/>
       <c r="AK3" s="15"/>
-      <c r="AL3" s="49" t="s">
+      <c r="AL3" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="AM3" s="49"/>
-      <c r="AN3" s="49"/>
-      <c r="AO3" s="49"/>
-      <c r="AP3" s="49"/>
-      <c r="AQ3" s="49"/>
-      <c r="AR3" s="49"/>
-      <c r="AS3" s="49"/>
-      <c r="AT3" s="49"/>
-      <c r="AU3" s="49"/>
-      <c r="AV3" s="49"/>
-      <c r="AW3" s="49"/>
-      <c r="AX3" s="49"/>
-      <c r="AY3" s="49"/>
-      <c r="AZ3" s="49"/>
-      <c r="BA3" s="49"/>
-      <c r="BB3" s="49"/>
-      <c r="BC3" s="49"/>
-      <c r="BD3" s="49"/>
-      <c r="BE3" s="49"/>
-      <c r="BF3" s="49"/>
-      <c r="BG3" s="49"/>
-      <c r="BH3" s="49"/>
-      <c r="BI3" s="49"/>
+      <c r="AM3" s="64"/>
+      <c r="AN3" s="64"/>
+      <c r="AO3" s="64"/>
+      <c r="AP3" s="64"/>
+      <c r="AQ3" s="64"/>
+      <c r="AR3" s="64"/>
+      <c r="AS3" s="64"/>
+      <c r="AT3" s="64"/>
+      <c r="AU3" s="64"/>
+      <c r="AV3" s="64"/>
+      <c r="AW3" s="64"/>
+      <c r="AX3" s="64"/>
+      <c r="AY3" s="64"/>
+      <c r="AZ3" s="64"/>
+      <c r="BA3" s="64"/>
+      <c r="BB3" s="64"/>
+      <c r="BC3" s="64"/>
+      <c r="BD3" s="64"/>
+      <c r="BE3" s="64"/>
+      <c r="BF3" s="64"/>
+      <c r="BG3" s="64"/>
+      <c r="BH3" s="64"/>
+      <c r="BI3" s="64"/>
       <c r="BJ3" s="8"/>
       <c r="BK3" s="8"/>
       <c r="BL3" s="8"/>
@@ -1825,77 +1823,77 @@
       <c r="A4" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="50"/>
-      <c r="D4" s="50"/>
-      <c r="E4" s="50"/>
-      <c r="F4" s="50" t="s">
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="50"/>
-      <c r="H4" s="50"/>
-      <c r="I4" s="50"/>
-      <c r="J4" s="50"/>
-      <c r="K4" s="50" t="s">
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
+      <c r="K4" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="L4" s="50"/>
-      <c r="M4" s="50"/>
-      <c r="N4" s="50"/>
-      <c r="O4" s="50"/>
-      <c r="P4" s="50"/>
-      <c r="Q4" s="50"/>
-      <c r="R4" s="50" t="s">
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
+      <c r="N4" s="47"/>
+      <c r="O4" s="47"/>
+      <c r="P4" s="47"/>
+      <c r="Q4" s="47"/>
+      <c r="R4" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="S4" s="50"/>
-      <c r="T4" s="50"/>
-      <c r="U4" s="50"/>
-      <c r="V4" s="50"/>
-      <c r="W4" s="50"/>
-      <c r="X4" s="50"/>
-      <c r="Y4" s="50"/>
-      <c r="Z4" s="50"/>
-      <c r="AA4" s="50"/>
-      <c r="AB4" s="50" t="s">
+      <c r="S4" s="47"/>
+      <c r="T4" s="47"/>
+      <c r="U4" s="47"/>
+      <c r="V4" s="47"/>
+      <c r="W4" s="47"/>
+      <c r="X4" s="47"/>
+      <c r="Y4" s="47"/>
+      <c r="Z4" s="47"/>
+      <c r="AA4" s="47"/>
+      <c r="AB4" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="AC4" s="50"/>
-      <c r="AD4" s="50"/>
-      <c r="AE4" s="50"/>
-      <c r="AF4" s="50"/>
-      <c r="AG4" s="50"/>
-      <c r="AH4" s="50"/>
-      <c r="AI4" s="50"/>
-      <c r="AJ4" s="50"/>
-      <c r="AK4" s="50"/>
-      <c r="AL4" s="50"/>
-      <c r="AM4" s="50" t="s">
+      <c r="AC4" s="47"/>
+      <c r="AD4" s="47"/>
+      <c r="AE4" s="47"/>
+      <c r="AF4" s="47"/>
+      <c r="AG4" s="47"/>
+      <c r="AH4" s="47"/>
+      <c r="AI4" s="47"/>
+      <c r="AJ4" s="47"/>
+      <c r="AK4" s="47"/>
+      <c r="AL4" s="47"/>
+      <c r="AM4" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="AN4" s="50"/>
-      <c r="AO4" s="50"/>
-      <c r="AP4" s="50"/>
-      <c r="AQ4" s="50"/>
-      <c r="AR4" s="50"/>
-      <c r="AS4" s="50"/>
-      <c r="AT4" s="50"/>
-      <c r="AU4" s="50"/>
-      <c r="AV4" s="50"/>
-      <c r="AW4" s="50"/>
-      <c r="AX4" s="50"/>
-      <c r="AY4" s="50"/>
-      <c r="AZ4" s="50"/>
-      <c r="BA4" s="50"/>
-      <c r="BB4" s="50"/>
-      <c r="BC4" s="50"/>
-      <c r="BD4" s="50"/>
-      <c r="BE4" s="50"/>
-      <c r="BF4" s="50"/>
-      <c r="BG4" s="50"/>
-      <c r="BH4" s="50"/>
+      <c r="AN4" s="47"/>
+      <c r="AO4" s="47"/>
+      <c r="AP4" s="47"/>
+      <c r="AQ4" s="47"/>
+      <c r="AR4" s="47"/>
+      <c r="AS4" s="47"/>
+      <c r="AT4" s="47"/>
+      <c r="AU4" s="47"/>
+      <c r="AV4" s="47"/>
+      <c r="AW4" s="47"/>
+      <c r="AX4" s="47"/>
+      <c r="AY4" s="47"/>
+      <c r="AZ4" s="47"/>
+      <c r="BA4" s="47"/>
+      <c r="BB4" s="47"/>
+      <c r="BC4" s="47"/>
+      <c r="BD4" s="47"/>
+      <c r="BE4" s="47"/>
+      <c r="BF4" s="47"/>
+      <c r="BG4" s="47"/>
+      <c r="BH4" s="47"/>
       <c r="BI4" s="36"/>
       <c r="BJ4" s="36"/>
       <c r="BK4" s="36"/>
@@ -1927,35 +1925,35 @@
       <c r="B5" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="55" t="s">
+      <c r="C5" s="49" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="55"/>
+      <c r="D5" s="49"/>
       <c r="E5" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="49" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="55"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="55"/>
-      <c r="J5" s="55"/>
-      <c r="K5" s="55" t="s">
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49" t="s">
         <v>82</v>
       </c>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="55" t="s">
+      <c r="L5" s="49"/>
+      <c r="M5" s="49"/>
+      <c r="N5" s="49" t="s">
         <v>90</v>
       </c>
-      <c r="O5" s="55"/>
-      <c r="P5" s="55"/>
-      <c r="Q5" s="55"/>
-      <c r="R5" s="55" t="s">
+      <c r="O5" s="49"/>
+      <c r="P5" s="49"/>
+      <c r="Q5" s="49"/>
+      <c r="R5" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="S5" s="55"/>
+      <c r="S5" s="49"/>
       <c r="T5" s="24" t="s">
         <v>29</v>
       </c>
@@ -1965,62 +1963,62 @@
       <c r="X5" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="Y5" s="55" t="s">
+      <c r="Y5" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="Z5" s="55"/>
-      <c r="AA5" s="55"/>
+      <c r="Z5" s="49"/>
+      <c r="AA5" s="49"/>
       <c r="AB5" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="AC5" s="75" t="s">
+      <c r="AC5" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="AD5" s="75"/>
-      <c r="AE5" s="55" t="s">
+      <c r="AD5" s="50"/>
+      <c r="AE5" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="AF5" s="55"/>
-      <c r="AG5" s="55" t="s">
+      <c r="AF5" s="49"/>
+      <c r="AG5" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="AH5" s="55"/>
-      <c r="AI5" s="55" t="s">
+      <c r="AH5" s="49"/>
+      <c r="AI5" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="AJ5" s="55"/>
-      <c r="AK5" s="55" t="s">
+      <c r="AJ5" s="49"/>
+      <c r="AK5" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="AL5" s="55"/>
-      <c r="AM5" s="55" t="s">
+      <c r="AL5" s="49"/>
+      <c r="AM5" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="AN5" s="55"/>
-      <c r="AO5" s="55"/>
-      <c r="AP5" s="55"/>
-      <c r="AQ5" s="55"/>
-      <c r="AR5" s="55"/>
-      <c r="AS5" s="55"/>
-      <c r="AT5" s="55" t="s">
+      <c r="AN5" s="49"/>
+      <c r="AO5" s="49"/>
+      <c r="AP5" s="49"/>
+      <c r="AQ5" s="49"/>
+      <c r="AR5" s="49"/>
+      <c r="AS5" s="49"/>
+      <c r="AT5" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="AU5" s="55"/>
-      <c r="AV5" s="55"/>
-      <c r="AW5" s="55"/>
-      <c r="AX5" s="51" t="s">
+      <c r="AU5" s="49"/>
+      <c r="AV5" s="49"/>
+      <c r="AW5" s="49"/>
+      <c r="AX5" s="73" t="s">
         <v>102</v>
       </c>
-      <c r="AY5" s="51"/>
-      <c r="AZ5" s="51"/>
-      <c r="BA5" s="51"/>
-      <c r="BB5" s="55"/>
-      <c r="BC5" s="55"/>
-      <c r="BD5" s="55"/>
-      <c r="BE5" s="55"/>
-      <c r="BF5" s="8"/>
-      <c r="BG5" s="8"/>
-      <c r="BH5" s="8"/>
+      <c r="AY5" s="73"/>
+      <c r="AZ5" s="73"/>
+      <c r="BA5" s="73"/>
+      <c r="BB5" s="49"/>
+      <c r="BC5" s="49"/>
+      <c r="BD5" s="49"/>
+      <c r="BE5" s="49"/>
+      <c r="BF5" s="49"/>
+      <c r="BG5" s="49"/>
+      <c r="BH5" s="49"/>
       <c r="BI5" s="8"/>
       <c r="BJ5" s="8"/>
       <c r="BK5" s="8"/>
@@ -2055,69 +2053,69 @@
       <c r="C6" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="72" t="s">
+      <c r="F6" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="72"/>
-      <c r="H6" s="72"/>
-      <c r="I6" s="72"/>
-      <c r="J6" s="72"/>
-      <c r="K6" s="72"/>
-      <c r="L6" s="72"/>
-      <c r="M6" s="72"/>
-      <c r="N6" s="72"/>
-      <c r="O6" s="72"/>
-      <c r="P6" s="72"/>
-      <c r="Q6" s="72" t="s">
+      <c r="G6" s="51"/>
+      <c r="H6" s="51"/>
+      <c r="I6" s="51"/>
+      <c r="J6" s="51"/>
+      <c r="K6" s="51"/>
+      <c r="L6" s="51"/>
+      <c r="M6" s="51"/>
+      <c r="N6" s="51"/>
+      <c r="O6" s="51"/>
+      <c r="P6" s="51"/>
+      <c r="Q6" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="R6" s="72"/>
-      <c r="S6" s="72"/>
-      <c r="T6" s="72"/>
-      <c r="U6" s="72"/>
-      <c r="V6" s="72"/>
-      <c r="W6" s="72"/>
-      <c r="X6" s="72"/>
-      <c r="Y6" s="72"/>
-      <c r="Z6" s="72"/>
-      <c r="AA6" s="72"/>
-      <c r="AB6" s="72" t="s">
+      <c r="R6" s="51"/>
+      <c r="S6" s="51"/>
+      <c r="T6" s="51"/>
+      <c r="U6" s="51"/>
+      <c r="V6" s="51"/>
+      <c r="W6" s="51"/>
+      <c r="X6" s="51"/>
+      <c r="Y6" s="51"/>
+      <c r="Z6" s="51"/>
+      <c r="AA6" s="51"/>
+      <c r="AB6" s="51" t="s">
         <v>44</v>
       </c>
-      <c r="AC6" s="72"/>
-      <c r="AD6" s="72"/>
-      <c r="AE6" s="72"/>
-      <c r="AF6" s="72"/>
-      <c r="AG6" s="72"/>
-      <c r="AH6" s="72"/>
-      <c r="AI6" s="72"/>
-      <c r="AJ6" s="72"/>
-      <c r="AK6" s="72"/>
-      <c r="AL6" s="72"/>
-      <c r="AM6" s="52" t="s">
+      <c r="AC6" s="51"/>
+      <c r="AD6" s="51"/>
+      <c r="AE6" s="51"/>
+      <c r="AF6" s="51"/>
+      <c r="AG6" s="51"/>
+      <c r="AH6" s="51"/>
+      <c r="AI6" s="51"/>
+      <c r="AJ6" s="51"/>
+      <c r="AK6" s="51"/>
+      <c r="AL6" s="51"/>
+      <c r="AM6" s="74" t="s">
         <v>100</v>
       </c>
-      <c r="AN6" s="53"/>
-      <c r="AO6" s="53"/>
-      <c r="AP6" s="53"/>
-      <c r="AQ6" s="53"/>
-      <c r="AR6" s="53"/>
-      <c r="AS6" s="53"/>
-      <c r="AT6" s="53"/>
-      <c r="AU6" s="53"/>
-      <c r="AV6" s="53"/>
-      <c r="AW6" s="53"/>
-      <c r="AX6" s="52"/>
-      <c r="AY6" s="53"/>
-      <c r="AZ6" s="53"/>
-      <c r="BA6" s="53"/>
-      <c r="BB6" s="53"/>
-      <c r="BC6" s="53"/>
-      <c r="BD6" s="53"/>
-      <c r="BE6" s="53"/>
-      <c r="BF6" s="53"/>
-      <c r="BG6" s="53"/>
-      <c r="BH6" s="53"/>
+      <c r="AN6" s="74"/>
+      <c r="AO6" s="74"/>
+      <c r="AP6" s="74"/>
+      <c r="AQ6" s="74"/>
+      <c r="AR6" s="74"/>
+      <c r="AS6" s="74"/>
+      <c r="AT6" s="74"/>
+      <c r="AU6" s="74"/>
+      <c r="AV6" s="74"/>
+      <c r="AW6" s="74"/>
+      <c r="AX6" s="74"/>
+      <c r="AY6" s="74"/>
+      <c r="AZ6" s="74"/>
+      <c r="BA6" s="74"/>
+      <c r="BB6" s="74"/>
+      <c r="BC6" s="74"/>
+      <c r="BD6" s="74"/>
+      <c r="BE6" s="74"/>
+      <c r="BF6" s="74"/>
+      <c r="BG6" s="74"/>
+      <c r="BH6" s="74"/>
       <c r="BI6" s="8"/>
       <c r="BJ6" s="8"/>
       <c r="BK6" s="8"/>
@@ -2146,78 +2144,81 @@
       <c r="A7" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="68" t="s">
+      <c r="B7" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
-      <c r="F7" s="54" t="s">
+      <c r="C7" s="60"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
-      <c r="I7" s="54"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="54"/>
-      <c r="L7" s="54"/>
-      <c r="M7" s="54"/>
-      <c r="N7" s="54"/>
-      <c r="O7" s="54"/>
-      <c r="P7" s="54"/>
-      <c r="Q7" s="73" t="s">
+      <c r="G7" s="48"/>
+      <c r="H7" s="48"/>
+      <c r="I7" s="48"/>
+      <c r="J7" s="48"/>
+      <c r="K7" s="48"/>
+      <c r="L7" s="48"/>
+      <c r="M7" s="48"/>
+      <c r="N7" s="48"/>
+      <c r="O7" s="48"/>
+      <c r="P7" s="48"/>
+      <c r="Q7" s="52" t="s">
         <v>48</v>
       </c>
-      <c r="R7" s="73"/>
-      <c r="S7" s="73"/>
-      <c r="T7" s="73"/>
-      <c r="U7" s="73"/>
-      <c r="V7" s="73"/>
-      <c r="W7" s="73"/>
-      <c r="X7" s="73"/>
-      <c r="Y7" s="54" t="s">
+      <c r="R7" s="52"/>
+      <c r="S7" s="52"/>
+      <c r="T7" s="52"/>
+      <c r="U7" s="52"/>
+      <c r="V7" s="52"/>
+      <c r="W7" s="52"/>
+      <c r="X7" s="52"/>
+      <c r="Y7" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="Z7" s="54"/>
-      <c r="AA7" s="54"/>
-      <c r="AB7" s="54"/>
-      <c r="AC7" s="54"/>
-      <c r="AD7" s="54"/>
-      <c r="AE7" s="54"/>
-      <c r="AF7" s="54"/>
-      <c r="AG7" s="54"/>
-      <c r="AH7" s="54" t="s">
+      <c r="Z7" s="48"/>
+      <c r="AA7" s="48"/>
+      <c r="AB7" s="48"/>
+      <c r="AC7" s="48"/>
+      <c r="AD7" s="48"/>
+      <c r="AE7" s="48"/>
+      <c r="AF7" s="48"/>
+      <c r="AG7" s="48"/>
+      <c r="AH7" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="AI7" s="54"/>
-      <c r="AJ7" s="54"/>
-      <c r="AK7" s="54"/>
-      <c r="AL7" s="54"/>
-      <c r="AM7" s="54"/>
-      <c r="AN7" s="54" t="s">
+      <c r="AI7" s="48"/>
+      <c r="AJ7" s="48"/>
+      <c r="AK7" s="48"/>
+      <c r="AL7" s="48"/>
+      <c r="AM7" s="48"/>
+      <c r="AN7" s="48" t="s">
         <v>51</v>
       </c>
-      <c r="AO7" s="54"/>
-      <c r="AP7" s="54"/>
-      <c r="AQ7" s="54"/>
-      <c r="AR7" s="54"/>
-      <c r="AS7" s="54"/>
-      <c r="AT7" s="54" t="s">
+      <c r="AO7" s="48"/>
+      <c r="AP7" s="48"/>
+      <c r="AQ7" s="48"/>
+      <c r="AR7" s="48"/>
+      <c r="AS7" s="48"/>
+      <c r="AT7" s="48" t="s">
         <v>52</v>
       </c>
-      <c r="AU7" s="54"/>
-      <c r="AV7" s="54"/>
-      <c r="AW7" s="54"/>
-      <c r="AX7" s="54" t="s">
+      <c r="AU7" s="48"/>
+      <c r="AV7" s="48"/>
+      <c r="AW7" s="48"/>
+      <c r="AX7" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="AY7" s="54"/>
-      <c r="AZ7" s="54"/>
-      <c r="BA7" s="54"/>
-      <c r="BB7" s="54"/>
-      <c r="BC7" s="54"/>
-      <c r="BD7" s="54"/>
-      <c r="BE7" s="54"/>
+      <c r="AY7" s="48"/>
+      <c r="AZ7" s="48"/>
+      <c r="BA7" s="48"/>
+      <c r="BB7" s="48"/>
+      <c r="BC7" s="48"/>
+      <c r="BD7" s="48"/>
+      <c r="BE7" s="48"/>
+      <c r="BF7" s="48"/>
+      <c r="BG7" s="48"/>
+      <c r="BH7" s="48"/>
     </row>
     <row r="8" spans="1:83" s="11" customFormat="1" ht="310.5" customHeight="1">
       <c r="A8" s="30" t="s">
@@ -2226,75 +2227,77 @@
       <c r="B8" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="57" t="s">
+      <c r="C8" s="66" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="57"/>
+      <c r="D8" s="66"/>
       <c r="E8" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="74" t="s">
+      <c r="F8" s="53" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="74"/>
-      <c r="H8" s="74"/>
-      <c r="I8" s="74"/>
-      <c r="J8" s="74"/>
-      <c r="K8" s="74"/>
-      <c r="L8" s="74"/>
-      <c r="M8" s="74"/>
-      <c r="N8" s="74"/>
-      <c r="O8" s="74"/>
-      <c r="P8" s="74"/>
+      <c r="G8" s="53"/>
+      <c r="H8" s="53"/>
+      <c r="I8" s="53"/>
+      <c r="J8" s="53"/>
+      <c r="K8" s="53"/>
+      <c r="L8" s="53"/>
+      <c r="M8" s="53"/>
+      <c r="N8" s="53"/>
+      <c r="O8" s="53"/>
+      <c r="P8" s="53"/>
       <c r="Q8" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="R8" s="62" t="s">
+      <c r="R8" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="S8" s="62"/>
+      <c r="S8" s="54"/>
       <c r="T8" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="U8" s="62" t="s">
+      <c r="U8" s="54" t="s">
         <v>61</v>
       </c>
-      <c r="V8" s="62"/>
-      <c r="Y8" s="60" t="s">
+      <c r="V8" s="54"/>
+      <c r="Y8" s="69" t="s">
         <v>62</v>
       </c>
-      <c r="Z8" s="60"/>
-      <c r="AA8" s="60"/>
-      <c r="AB8" s="60"/>
+      <c r="Z8" s="69"/>
+      <c r="AA8" s="69"/>
+      <c r="AB8" s="69"/>
       <c r="AC8" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="AD8" s="62" t="s">
+      <c r="AD8" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="AE8" s="62"/>
-      <c r="AF8" s="62" t="s">
+      <c r="AE8" s="54"/>
+      <c r="AF8" s="54" t="s">
         <v>83</v>
       </c>
-      <c r="AG8" s="62"/>
-      <c r="AH8" s="62"/>
-      <c r="AI8" s="62"/>
-      <c r="AJ8" s="62" t="s">
+      <c r="AG8" s="54"/>
+      <c r="AH8" s="54"/>
+      <c r="AI8" s="54"/>
+      <c r="AJ8" s="54" t="s">
         <v>65</v>
       </c>
-      <c r="AK8" s="62"/>
-      <c r="AL8" s="62"/>
-      <c r="AM8" s="62" t="s">
+      <c r="AK8" s="54"/>
+      <c r="AL8" s="54"/>
+      <c r="AM8" s="54" t="s">
         <v>66</v>
       </c>
-      <c r="AN8" s="62"/>
-      <c r="AO8" s="62"/>
-      <c r="BC8" s="8"/>
-      <c r="BD8" s="8"/>
-      <c r="BE8" s="8"/>
-      <c r="BF8" s="8"/>
-      <c r="BG8" s="8"/>
-      <c r="BH8" s="8"/>
+      <c r="AN8" s="54"/>
+      <c r="AO8" s="54"/>
+      <c r="BA8" s="75"/>
+      <c r="BB8" s="75"/>
+      <c r="BC8" s="75"/>
+      <c r="BD8" s="75"/>
+      <c r="BE8" s="75"/>
+      <c r="BF8" s="75"/>
+      <c r="BG8" s="75"/>
+      <c r="BH8" s="75"/>
       <c r="BI8" s="8"/>
       <c r="BJ8" s="8"/>
       <c r="BK8" s="8"/>
@@ -2324,73 +2327,67 @@
         <v>67</v>
       </c>
       <c r="B9" s="9"/>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="48"/>
-      <c r="E9" s="59" t="s">
+      <c r="D9" s="46"/>
+      <c r="E9" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
-      <c r="M9" s="48" t="s">
+      <c r="F9" s="68"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="68"/>
+      <c r="I9" s="68"/>
+      <c r="J9" s="68"/>
+      <c r="K9" s="68"/>
+      <c r="L9" s="68"/>
+      <c r="M9" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="N9" s="48"/>
-      <c r="O9" s="48"/>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="48"/>
-      <c r="R9" s="48"/>
-      <c r="S9" s="48"/>
-      <c r="T9" s="48"/>
-      <c r="U9" s="48" t="s">
+      <c r="N9" s="46"/>
+      <c r="O9" s="46"/>
+      <c r="P9" s="46"/>
+      <c r="Q9" s="46"/>
+      <c r="R9" s="46"/>
+      <c r="S9" s="46"/>
+      <c r="T9" s="46"/>
+      <c r="U9" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="V9" s="48"/>
-      <c r="W9" s="48"/>
-      <c r="X9" s="48"/>
-      <c r="Y9" s="48"/>
-      <c r="Z9" s="48"/>
-      <c r="AA9" s="48"/>
-      <c r="AB9" s="48"/>
-      <c r="AC9" s="48" t="s">
+      <c r="V9" s="46"/>
+      <c r="W9" s="46"/>
+      <c r="X9" s="46"/>
+      <c r="Y9" s="46"/>
+      <c r="Z9" s="46"/>
+      <c r="AA9" s="46"/>
+      <c r="AB9" s="46"/>
+      <c r="AC9" s="46" t="s">
         <v>70</v>
       </c>
-      <c r="AD9" s="48"/>
-      <c r="AE9" s="48"/>
-      <c r="AF9" s="48"/>
-      <c r="AG9" s="48"/>
-      <c r="AH9" s="48"/>
-      <c r="AI9" s="48"/>
-      <c r="AJ9" s="48"/>
-      <c r="AK9" s="48"/>
-      <c r="AN9" s="48" t="s">
+      <c r="AD9" s="46"/>
+      <c r="AE9" s="46"/>
+      <c r="AF9" s="46"/>
+      <c r="AG9" s="46"/>
+      <c r="AH9" s="46"/>
+      <c r="AI9" s="46"/>
+      <c r="AJ9" s="46"/>
+      <c r="AK9" s="46"/>
+      <c r="AN9" s="46" t="s">
         <v>101</v>
       </c>
-      <c r="AO9" s="48"/>
-      <c r="AP9" s="48"/>
-      <c r="AQ9" s="48"/>
-      <c r="AR9" s="48"/>
-      <c r="AS9" s="48"/>
-      <c r="AT9" s="48"/>
-      <c r="AU9" s="48"/>
-      <c r="AY9" s="48" t="s">
+      <c r="AO9" s="46"/>
+      <c r="AP9" s="46"/>
+      <c r="AQ9" s="46"/>
+      <c r="AR9" s="46"/>
+      <c r="AS9" s="46"/>
+      <c r="AT9" s="46"/>
+      <c r="AU9" s="46"/>
+      <c r="AY9" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="AZ9" s="48"/>
-      <c r="BA9" s="48"/>
-      <c r="BB9" s="48"/>
-      <c r="BC9" s="8"/>
-      <c r="BD9" s="8"/>
-      <c r="BE9" s="8"/>
-      <c r="BF9" s="8"/>
-      <c r="BG9" s="8"/>
-      <c r="BH9" s="8"/>
+      <c r="AZ9" s="46"/>
+      <c r="BA9" s="46"/>
+      <c r="BB9" s="46"/>
       <c r="BI9" s="8"/>
       <c r="BJ9" s="8"/>
       <c r="BK9" s="8"/>
@@ -2419,11 +2416,11 @@
       <c r="A10" s="39" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="58" t="s">
+      <c r="B10" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
+      <c r="C10" s="67"/>
+      <c r="D10" s="67"/>
       <c r="E10" s="35" t="s">
         <v>97</v>
       </c>
@@ -2458,10 +2455,10 @@
       <c r="AE10" s="45"/>
       <c r="AF10" s="45"/>
       <c r="AG10" s="45"/>
-      <c r="AI10" s="61" t="s">
+      <c r="AI10" s="70" t="s">
         <v>81</v>
       </c>
-      <c r="AJ10" s="61"/>
+      <c r="AJ10" s="70"/>
       <c r="AK10" s="45" t="s">
         <v>94</v>
       </c>
@@ -2491,7 +2488,6 @@
       <c r="BE10" s="45"/>
       <c r="BF10" s="45"/>
       <c r="BG10" s="45"/>
-      <c r="BH10" s="8"/>
       <c r="BI10" s="8"/>
       <c r="BJ10" s="8"/>
       <c r="BK10" s="8"/>
@@ -2517,11 +2513,11 @@
       <c r="CE10" s="8"/>
     </row>
     <row r="11" spans="1:83" ht="26.25" customHeight="1">
-      <c r="A11" s="56" t="s">
+      <c r="A11" s="65" t="s">
         <v>75</v>
       </c>
-      <c r="B11" s="56"/>
-      <c r="C11" s="56"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
       <c r="D11" s="38"/>
       <c r="E11" s="38"/>
     </row>
@@ -2549,33 +2545,40 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="75">
-    <mergeCell ref="AN10:AW10"/>
-    <mergeCell ref="AN9:AU9"/>
-    <mergeCell ref="R4:AA4"/>
-    <mergeCell ref="AH7:AM7"/>
-    <mergeCell ref="AM6:AW6"/>
-    <mergeCell ref="AT5:AW5"/>
-    <mergeCell ref="AM5:AS5"/>
-    <mergeCell ref="AC5:AD5"/>
-    <mergeCell ref="AE5:AF5"/>
-    <mergeCell ref="AG5:AH5"/>
-    <mergeCell ref="R5:S5"/>
-    <mergeCell ref="Q6:AA6"/>
-    <mergeCell ref="AN7:AS7"/>
-    <mergeCell ref="AT7:AW7"/>
-    <mergeCell ref="F7:P7"/>
-    <mergeCell ref="Q7:X7"/>
-    <mergeCell ref="Y7:AG7"/>
-    <mergeCell ref="F8:P8"/>
-    <mergeCell ref="AI5:AJ5"/>
-    <mergeCell ref="AB6:AL6"/>
-    <mergeCell ref="U8:V8"/>
-    <mergeCell ref="AK5:AL5"/>
-    <mergeCell ref="AJ8:AL8"/>
-    <mergeCell ref="R8:S8"/>
-    <mergeCell ref="AD8:AE8"/>
-    <mergeCell ref="AF8:AI8"/>
+  <mergeCells count="74">
+    <mergeCell ref="AX10:BG10"/>
+    <mergeCell ref="AX1:BH1"/>
+    <mergeCell ref="AY9:BB9"/>
+    <mergeCell ref="AX3:BI3"/>
+    <mergeCell ref="AX4:BH4"/>
+    <mergeCell ref="AX5:BA5"/>
+    <mergeCell ref="AX7:BA7"/>
+    <mergeCell ref="AM6:BH6"/>
+    <mergeCell ref="BB5:BH5"/>
+    <mergeCell ref="BB7:BH7"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="AC9:AK9"/>
+    <mergeCell ref="U9:AB9"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="R10:T10"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="M9:T9"/>
+    <mergeCell ref="J10:P10"/>
+    <mergeCell ref="E9:L9"/>
+    <mergeCell ref="U10:AA10"/>
+    <mergeCell ref="AC10:AG10"/>
+    <mergeCell ref="Y8:AB8"/>
+    <mergeCell ref="AK10:AM10"/>
+    <mergeCell ref="AI10:AJ10"/>
+    <mergeCell ref="AM8:AO8"/>
+    <mergeCell ref="AB1:AL1"/>
+    <mergeCell ref="AB3:AF3"/>
+    <mergeCell ref="AB4:AL4"/>
+    <mergeCell ref="AK2:AL2"/>
+    <mergeCell ref="AM1:AW1"/>
+    <mergeCell ref="AM4:AW4"/>
+    <mergeCell ref="AL3:AW3"/>
     <mergeCell ref="F1:P1"/>
     <mergeCell ref="Q1:AA1"/>
     <mergeCell ref="B1:E1"/>
@@ -2592,39 +2595,31 @@
     <mergeCell ref="K4:Q4"/>
     <mergeCell ref="F6:P6"/>
     <mergeCell ref="F4:J4"/>
-    <mergeCell ref="AB1:AL1"/>
-    <mergeCell ref="AB3:AF3"/>
-    <mergeCell ref="AB4:AL4"/>
-    <mergeCell ref="AK2:AL2"/>
-    <mergeCell ref="AM1:AW1"/>
-    <mergeCell ref="AM4:AW4"/>
-    <mergeCell ref="AL3:AW3"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="AC9:AK9"/>
-    <mergeCell ref="U9:AB9"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="R10:T10"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="M9:T9"/>
-    <mergeCell ref="J10:P10"/>
-    <mergeCell ref="E9:L9"/>
-    <mergeCell ref="U10:AA10"/>
-    <mergeCell ref="AC10:AG10"/>
-    <mergeCell ref="Y8:AB8"/>
-    <mergeCell ref="AK10:AM10"/>
-    <mergeCell ref="AI10:AJ10"/>
-    <mergeCell ref="AM8:AO8"/>
-    <mergeCell ref="AX10:BG10"/>
-    <mergeCell ref="AX1:BH1"/>
-    <mergeCell ref="AY9:BB9"/>
-    <mergeCell ref="AX3:BI3"/>
-    <mergeCell ref="AX4:BH4"/>
-    <mergeCell ref="AX5:BA5"/>
-    <mergeCell ref="AX6:BH6"/>
-    <mergeCell ref="AX7:BA7"/>
-    <mergeCell ref="BB5:BE5"/>
-    <mergeCell ref="BB7:BE7"/>
+    <mergeCell ref="F7:P7"/>
+    <mergeCell ref="Q7:X7"/>
+    <mergeCell ref="Y7:AG7"/>
+    <mergeCell ref="F8:P8"/>
+    <mergeCell ref="AI5:AJ5"/>
+    <mergeCell ref="AB6:AL6"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="AK5:AL5"/>
+    <mergeCell ref="AJ8:AL8"/>
+    <mergeCell ref="R8:S8"/>
+    <mergeCell ref="AD8:AE8"/>
+    <mergeCell ref="AF8:AI8"/>
+    <mergeCell ref="AN10:AW10"/>
+    <mergeCell ref="AN9:AU9"/>
+    <mergeCell ref="R4:AA4"/>
+    <mergeCell ref="AH7:AM7"/>
+    <mergeCell ref="AT5:AW5"/>
+    <mergeCell ref="AM5:AS5"/>
+    <mergeCell ref="AC5:AD5"/>
+    <mergeCell ref="AE5:AF5"/>
+    <mergeCell ref="AG5:AH5"/>
+    <mergeCell ref="R5:S5"/>
+    <mergeCell ref="Q6:AA6"/>
+    <mergeCell ref="AN7:AS7"/>
+    <mergeCell ref="AT7:AW7"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="27" orientation="landscape" r:id="rId1"/>

</xml_diff>